<commit_message>
refactor: improve label text rendering
</commit_message>
<xml_diff>
--- a/input/demo_products.xlsx
+++ b/input/demo_products.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">article</t>
   </si>
@@ -34,6 +34,9 @@
     <t xml:space="preserve">price</t>
   </si>
   <si>
+    <t xml:space="preserve">currency</t>
+  </si>
+  <si>
     <t xml:space="preserve">227701</t>
   </si>
   <si>
@@ -43,6 +46,9 @@
     <t xml:space="preserve">40(p)</t>
   </si>
   <si>
+    <t xml:space="preserve">ГРН</t>
+  </si>
+  <si>
     <t xml:space="preserve">227702</t>
   </si>
   <si>
@@ -52,6 +58,9 @@
     <t xml:space="preserve">41(p)</t>
   </si>
   <si>
+    <t xml:space="preserve">USD</t>
+  </si>
+  <si>
     <t xml:space="preserve">227703</t>
   </si>
   <si>
@@ -59,6 +68,9 @@
   </si>
   <si>
     <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR</t>
   </si>
   <si>
     <t xml:space="preserve">227704</t>
@@ -165,8 +177,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
@@ -186,58 +198,70 @@
       <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="0" t="n">
         <v>9790</v>
       </c>
+      <c r="E2" s="0" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="0" t="n">
         <v>10250</v>
       </c>
+      <c r="E3" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4" s="0" t="n">
         <v>8450</v>
       </c>
+      <c r="E4" s="0" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D5" s="0" t="n">
         <v>12500</v>

</xml_diff>

<commit_message>
refactor: add configurable Excel column mapping
</commit_message>
<xml_diff>
--- a/input/demo_products.xlsx
+++ b/input/demo_products.xlsx
@@ -20,21 +20,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
-  <si>
-    <t xml:space="preserve">article</t>
-  </si>
-  <si>
-    <t xml:space="preserve">name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">currency</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+  <si>
+    <t xml:space="preserve">Артикул</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Название</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Размер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Валюта</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2601-BR-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giovanna 2601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ГРН</t>
   </si>
   <si>
     <t xml:space="preserve">227701</t>
@@ -44,9 +53,6 @@
   </si>
   <si>
     <t xml:space="preserve">40(p)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ГРН</t>
   </si>
   <si>
     <t xml:space="preserve">227702</t>
@@ -155,9 +161,13 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -177,7 +187,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -202,71 +212,89 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>10990</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="0" t="n">
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="0" t="n">
         <v>9790</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="0" t="s">
+      <c r="E3" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="B4" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="0" t="n">
         <v>10250</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="0" t="s">
+      <c r="E4" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="0" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="B5" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="0" t="n">
         <v>8450</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="0" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="B6" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="0" t="n">
         <v>12500</v>
       </c>
     </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
feat: support configurable barcode column mapping
</commit_message>
<xml_diff>
--- a/input/demo_products.xlsx
+++ b/input/demo_products.xlsx
@@ -20,12 +20,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t xml:space="preserve">Артикул</t>
   </si>
   <si>
     <t xml:space="preserve">Название</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Штрихкод</t>
   </si>
   <si>
     <t xml:space="preserve">Размер</t>
@@ -187,7 +190,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -195,7 +198,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
@@ -211,86 +214,89 @@
       <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="E2" s="0" t="n">
         <v>10990</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>7</v>
+      <c r="F2" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>9790</v>
+      </c>
+      <c r="F3" s="0" t="s">
         <v>8</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>9790</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="0" t="n">
         <v>10250</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>14</v>
+      <c r="F4" s="0" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="0" t="n">
         <v>8450</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>18</v>
+      <c r="F5" s="0" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="0" t="n">
         <v>12500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: add requirements file and update readme
</commit_message>
<xml_diff>
--- a/input/demo_products.xlsx
+++ b/input/demo_products.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">Артикул</t>
   </si>
@@ -40,55 +40,13 @@
     <t xml:space="preserve">Валюта</t>
   </si>
   <si>
-    <t xml:space="preserve">2601-BR-37</t>
+    <t xml:space="preserve">2xx1-BR-37</t>
   </si>
   <si>
     <t xml:space="preserve">Giovanna 2601</t>
   </si>
   <si>
-    <t xml:space="preserve">ГРН</t>
-  </si>
-  <si>
-    <t xml:space="preserve">227701</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICEBERG белый</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40(p)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">227702</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICEBERG чёрный</t>
-  </si>
-  <si>
-    <t xml:space="preserve">41(p)</t>
-  </si>
-  <si>
     <t xml:space="preserve">USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">227703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COSMO light jacket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EUR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">227704</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Winter boots premium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">43</t>
   </si>
 </sst>
 </file>
@@ -229,75 +187,10 @@
         <v>37</v>
       </c>
       <c r="E2" s="0" t="n">
-        <v>10990</v>
+        <v>199</v>
       </c>
       <c r="F2" s="0" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="0" t="n">
-        <v>9790</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="0" t="n">
-        <v>10250</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="0" t="n">
-        <v>8450</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="0" t="n">
-        <v>12500</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>